<commit_message>
auto: excel 02/07/2026 15:04
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333585B6-18B0-4CD3-821B-1BC184CB8E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8A9E13-C51B-4ABC-83D7-F4761622C5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="940">
   <si>
     <t>CONTENTOR</t>
   </si>
@@ -2925,6 +2925,9 @@
   </si>
   <si>
     <t>NÃO</t>
+  </si>
+  <si>
+    <t>sim</t>
   </si>
 </sst>
 </file>
@@ -19139,7 +19142,7 @@
         <v>46270</v>
       </c>
       <c r="I59" s="29" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="J59" s="29"/>
       <c r="K59" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:11
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8A9E13-C51B-4ABC-83D7-F4761622C5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE195610-BCEC-4745-A72B-432D1E263FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -19187,7 +19187,7 @@
         <v>46254</v>
       </c>
       <c r="I60" s="29" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="J60" s="29"/>
       <c r="K60" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:12
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE195610-BCEC-4745-A72B-432D1E263FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590E72E5-92CA-4489-81AB-BB6681DB62B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="940">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="939">
   <si>
     <t>CONTENTOR</t>
   </si>
@@ -2925,9 +2925,6 @@
   </si>
   <si>
     <t>NÃO</t>
-  </si>
-  <si>
-    <t>sim</t>
   </si>
 </sst>
 </file>
@@ -19141,8 +19138,8 @@
       <c r="H59" s="29">
         <v>46270</v>
       </c>
-      <c r="I59" s="29" t="s">
-        <v>939</v>
+      <c r="I59" s="33" t="s">
+        <v>937</v>
       </c>
       <c r="J59" s="29"/>
       <c r="K59" s="14"/>
@@ -19186,8 +19183,8 @@
       <c r="H60" s="29">
         <v>46254</v>
       </c>
-      <c r="I60" s="29" t="s">
-        <v>939</v>
+      <c r="I60" s="33" t="s">
+        <v>937</v>
       </c>
       <c r="J60" s="29"/>
       <c r="K60" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:19
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590E72E5-92CA-4489-81AB-BB6681DB62B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F924BA13-A01A-4BEF-A737-7EB2774F11ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -19093,8 +19093,8 @@
       <c r="H58" s="29">
         <v>46247</v>
       </c>
-      <c r="I58" s="29" t="s">
-        <v>938</v>
+      <c r="I58" s="33" t="s">
+        <v>937</v>
       </c>
       <c r="J58" s="29"/>
       <c r="K58" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:31
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F924BA13-A01A-4BEF-A737-7EB2774F11ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546092F4-A1D9-4695-A12E-5FBD79805E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -19093,8 +19093,8 @@
       <c r="H58" s="29">
         <v>46247</v>
       </c>
-      <c r="I58" s="33" t="s">
-        <v>937</v>
+      <c r="I58" s="29" t="s">
+        <v>938</v>
       </c>
       <c r="J58" s="29"/>
       <c r="K58" s="14"/>
@@ -19138,8 +19138,8 @@
       <c r="H59" s="29">
         <v>46270</v>
       </c>
-      <c r="I59" s="33" t="s">
-        <v>937</v>
+      <c r="I59" s="29" t="s">
+        <v>938</v>
       </c>
       <c r="J59" s="29"/>
       <c r="K59" s="14"/>
@@ -19183,8 +19183,8 @@
       <c r="H60" s="29">
         <v>46254</v>
       </c>
-      <c r="I60" s="33" t="s">
-        <v>937</v>
+      <c r="I60" s="29" t="s">
+        <v>938</v>
       </c>
       <c r="J60" s="29"/>
       <c r="K60" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:32
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546092F4-A1D9-4695-A12E-5FBD79805E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37069CF6-5545-40B5-9BD0-97D8FE5E170A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -18868,8 +18868,8 @@
       <c r="H53" s="29">
         <v>46234</v>
       </c>
-      <c r="I53" s="29" t="s">
-        <v>938</v>
+      <c r="I53" s="33" t="s">
+        <v>937</v>
       </c>
       <c r="J53" s="29"/>
       <c r="K53" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:43
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37069CF6-5545-40B5-9BD0-97D8FE5E170A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A52506E-8D83-4A21-9886-8B376CFDE98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -18868,8 +18868,8 @@
       <c r="H53" s="29">
         <v>46234</v>
       </c>
-      <c r="I53" s="33" t="s">
-        <v>937</v>
+      <c r="I53" s="29" t="s">
+        <v>938</v>
       </c>
       <c r="J53" s="29"/>
       <c r="K53" s="14"/>

</xml_diff>

<commit_message>
auto: excel 02/07/2026 15:46
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A52506E-8D83-4A21-9886-8B376CFDE98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF398E94-2485-4CDF-A16B-E0B280425E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -18913,8 +18913,8 @@
       <c r="H54" s="29">
         <v>46240</v>
       </c>
-      <c r="I54" s="29" t="s">
-        <v>938</v>
+      <c r="I54" s="33" t="s">
+        <v>937</v>
       </c>
       <c r="J54" s="29"/>
       <c r="K54" s="14" t="s">

</xml_diff>

<commit_message>
auto: excel 02/07/2026 16:05
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF398E94-2485-4CDF-A16B-E0B280425E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1267B62E-16DC-4BE7-B4F0-C0FCCDC0FF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -18913,8 +18913,8 @@
       <c r="H54" s="29">
         <v>46240</v>
       </c>
-      <c r="I54" s="33" t="s">
-        <v>937</v>
+      <c r="I54" s="29" t="s">
+        <v>938</v>
       </c>
       <c r="J54" s="29"/>
       <c r="K54" s="14" t="s">

</xml_diff>

<commit_message>
auto: excel 02/07/2026 16:30
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1267B62E-16DC-4BE7-B4F0-C0FCCDC0FF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3737A645-C4DC-485C-A486-E1A9FC7AA1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -18914,7 +18914,7 @@
         <v>46240</v>
       </c>
       <c r="I54" s="29" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="J54" s="29"/>
       <c r="K54" s="14" t="s">

</xml_diff>

<commit_message>
auto: excel 02/07/2026 17:00
</commit_message>
<xml_diff>
--- a/CONTENTORES-MATERIAL Final-2026.xlsx
+++ b/CONTENTORES-MATERIAL Final-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Polho\iCloudDrive2\iCloudDrive\Gestao de compras\cowork\contentores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3737A645-C4DC-485C-A486-E1A9FC7AA1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA36F6A-D191-4A73-8910-FE9020719062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2325" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{932CD236-D129-441F-BCD4-FAC853A5E9F7}"/>
   </bookViews>
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2342" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2402" uniqueCount="940">
   <si>
     <t>CONTENTOR</t>
   </si>
@@ -2925,6 +2925,9 @@
   </si>
   <si>
     <t>NÃO</t>
+  </si>
+  <si>
+    <t>AVISO</t>
   </si>
 </sst>
 </file>
@@ -16389,7 +16392,9 @@
       <c r="I1" s="7" t="s">
         <v>936</v>
       </c>
-      <c r="J1" s="7"/>
+      <c r="J1" s="7" t="s">
+        <v>939</v>
+      </c>
       <c r="K1" s="8" t="s">
         <v>55</v>
       </c>
@@ -16452,7 +16457,9 @@
       <c r="I2" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J2" s="33"/>
+      <c r="J2" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K2" s="34"/>
       <c r="L2" s="34">
         <v>46030</v>
@@ -16499,7 +16506,9 @@
       <c r="I3" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J3" s="33"/>
+      <c r="J3" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K3" s="34"/>
       <c r="L3" s="34">
         <v>46029</v>
@@ -16546,7 +16555,9 @@
       <c r="I4" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J4" s="33"/>
+      <c r="J4" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K4" s="34"/>
       <c r="L4" s="34">
         <v>46028</v>
@@ -16593,7 +16604,9 @@
       <c r="I5" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J5" s="33"/>
+      <c r="J5" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K5" s="34"/>
       <c r="L5" s="34">
         <v>46036</v>
@@ -16640,7 +16653,9 @@
       <c r="I6" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J6" s="33"/>
+      <c r="J6" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K6" s="34"/>
       <c r="L6" s="34">
         <v>46037</v>
@@ -16685,7 +16700,9 @@
       <c r="I7" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J7" s="33"/>
+      <c r="J7" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K7" s="34"/>
       <c r="L7" s="34">
         <v>46038</v>
@@ -16730,7 +16747,9 @@
       <c r="I8" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J8" s="33"/>
+      <c r="J8" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K8" s="34"/>
       <c r="L8" s="34">
         <v>46041</v>
@@ -16777,7 +16796,9 @@
       <c r="I9" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J9" s="33"/>
+      <c r="J9" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K9" s="34"/>
       <c r="L9" s="34">
         <v>46037</v>
@@ -16824,7 +16845,9 @@
       <c r="I10" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J10" s="33"/>
+      <c r="J10" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K10" s="34"/>
       <c r="L10" s="34">
         <v>46038</v>
@@ -16871,7 +16894,9 @@
       <c r="I11" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J11" s="33"/>
+      <c r="J11" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K11" s="34"/>
       <c r="L11" s="34">
         <v>46044</v>
@@ -16918,7 +16943,9 @@
       <c r="I12" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J12" s="33"/>
+      <c r="J12" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K12" s="34"/>
       <c r="L12" s="34">
         <v>46042</v>
@@ -16967,7 +16994,9 @@
       <c r="I13" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J13" s="33"/>
+      <c r="J13" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K13" s="34"/>
       <c r="L13" s="34">
         <v>46045</v>
@@ -17016,7 +17045,9 @@
       <c r="I14" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J14" s="33"/>
+      <c r="J14" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K14" s="34"/>
       <c r="L14" s="34">
         <v>46050</v>
@@ -17063,7 +17094,9 @@
       <c r="I15" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J15" s="33"/>
+      <c r="J15" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K15" s="34"/>
       <c r="L15" s="34">
         <v>46051</v>
@@ -17110,7 +17143,9 @@
       <c r="I16" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J16" s="33"/>
+      <c r="J16" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K16" s="34"/>
       <c r="L16" s="34">
         <v>46051</v>
@@ -17157,7 +17192,9 @@
       <c r="I17" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J17" s="33"/>
+      <c r="J17" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K17" s="34" t="s">
         <v>306</v>
       </c>
@@ -17208,7 +17245,9 @@
       <c r="I18" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J18" s="33"/>
+      <c r="J18" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K18" s="34"/>
       <c r="L18" s="34">
         <v>46064</v>
@@ -17257,7 +17296,9 @@
       <c r="I19" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J19" s="33"/>
+      <c r="J19" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K19" s="34"/>
       <c r="L19" s="34">
         <v>46072</v>
@@ -17304,7 +17345,9 @@
       <c r="I20" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J20" s="33"/>
+      <c r="J20" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K20" s="34"/>
       <c r="L20" s="34">
         <v>46073</v>
@@ -17351,7 +17394,9 @@
       <c r="I21" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J21" s="33"/>
+      <c r="J21" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K21" s="34"/>
       <c r="L21" s="34">
         <v>46071</v>
@@ -17398,7 +17443,9 @@
       <c r="I22" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J22" s="33"/>
+      <c r="J22" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K22" s="34"/>
       <c r="L22" s="34">
         <v>46076</v>
@@ -17445,7 +17492,9 @@
       <c r="I23" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J23" s="33"/>
+      <c r="J23" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K23" s="34"/>
       <c r="L23" s="34">
         <v>46076</v>
@@ -17494,7 +17543,9 @@
       <c r="I24" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J24" s="33"/>
+      <c r="J24" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K24" s="34"/>
       <c r="L24" s="34">
         <v>46077</v>
@@ -17541,7 +17592,9 @@
       <c r="I25" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J25" s="33"/>
+      <c r="J25" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K25" s="34"/>
       <c r="L25" s="34">
         <v>46076</v>
@@ -17588,7 +17641,9 @@
       <c r="I26" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J26" s="33"/>
+      <c r="J26" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K26" s="34"/>
       <c r="L26" s="34">
         <v>46078</v>
@@ -17635,7 +17690,9 @@
       <c r="I27" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J27" s="33"/>
+      <c r="J27" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K27" s="34"/>
       <c r="L27" s="34">
         <v>46078</v>
@@ -17682,7 +17739,9 @@
       <c r="I28" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J28" s="33"/>
+      <c r="J28" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K28" s="34"/>
       <c r="L28" s="34">
         <v>46097</v>
@@ -17729,7 +17788,9 @@
       <c r="I29" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J29" s="33"/>
+      <c r="J29" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K29" s="34"/>
       <c r="L29" s="34">
         <v>46099</v>
@@ -17774,7 +17835,9 @@
       <c r="I30" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J30" s="33"/>
+      <c r="J30" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K30" s="34"/>
       <c r="L30" s="34">
         <v>46099</v>
@@ -17821,7 +17884,9 @@
       <c r="I31" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J31" s="33"/>
+      <c r="J31" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K31" s="34"/>
       <c r="L31" s="34">
         <v>46099</v>
@@ -17868,7 +17933,9 @@
       <c r="I32" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J32" s="33"/>
+      <c r="J32" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K32" s="34"/>
       <c r="L32" s="34">
         <v>46100</v>
@@ -17915,7 +17982,9 @@
       <c r="I33" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J33" s="33"/>
+      <c r="J33" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K33" s="34"/>
       <c r="L33" s="34">
         <v>46101</v>
@@ -17962,7 +18031,9 @@
       <c r="I34" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J34" s="33"/>
+      <c r="J34" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K34" s="34"/>
       <c r="L34" s="34">
         <v>46098</v>
@@ -18009,7 +18080,9 @@
       <c r="I35" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J35" s="33"/>
+      <c r="J35" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K35" s="34"/>
       <c r="L35" s="34">
         <v>46119</v>
@@ -18058,7 +18131,9 @@
       <c r="I36" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J36" s="33"/>
+      <c r="J36" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K36" s="34"/>
       <c r="L36" s="34">
         <v>46125</v>
@@ -18107,7 +18182,9 @@
       <c r="I37" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J37" s="33"/>
+      <c r="J37" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K37" s="34"/>
       <c r="L37" s="34">
         <v>46128</v>
@@ -18154,7 +18231,9 @@
       <c r="I38" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J38" s="33"/>
+      <c r="J38" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K38" s="34"/>
       <c r="L38" s="34">
         <v>46132</v>
@@ -18201,7 +18280,9 @@
       <c r="I39" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J39" s="33"/>
+      <c r="J39" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K39" s="34"/>
       <c r="L39" s="34">
         <v>46129</v>
@@ -18248,7 +18329,9 @@
       <c r="I40" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J40" s="33"/>
+      <c r="J40" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K40" s="34"/>
       <c r="L40" s="34">
         <v>46133</v>
@@ -18295,7 +18378,9 @@
       <c r="I41" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J41" s="33"/>
+      <c r="J41" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K41" s="34"/>
       <c r="L41" s="34">
         <v>46134</v>
@@ -18342,7 +18427,9 @@
       <c r="I42" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J42" s="33"/>
+      <c r="J42" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K42" s="34"/>
       <c r="L42" s="34">
         <v>46176</v>
@@ -18391,7 +18478,9 @@
       <c r="I43" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J43" s="33"/>
+      <c r="J43" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K43" s="34"/>
       <c r="L43" s="34">
         <v>46182</v>
@@ -18440,7 +18529,9 @@
       <c r="I44" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J44" s="33"/>
+      <c r="J44" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K44" s="34"/>
       <c r="L44" s="34">
         <v>46184</v>
@@ -18487,7 +18578,9 @@
       <c r="I45" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J45" s="33"/>
+      <c r="J45" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K45" s="34"/>
       <c r="L45" s="34">
         <v>46182</v>
@@ -18534,7 +18627,9 @@
       <c r="I46" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J46" s="33"/>
+      <c r="J46" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K46" s="34"/>
       <c r="L46" s="34">
         <v>46196</v>
@@ -18581,7 +18676,9 @@
       <c r="I47" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J47" s="33"/>
+      <c r="J47" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K47" s="34"/>
       <c r="L47" s="34">
         <v>46202</v>
@@ -18628,7 +18725,9 @@
       <c r="I48" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J48" s="33"/>
+      <c r="J48" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K48" s="34" t="s">
         <v>570</v>
       </c>
@@ -18677,7 +18776,9 @@
       <c r="I49" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J49" s="33"/>
+      <c r="J49" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K49" s="34"/>
       <c r="L49" s="34">
         <v>46202</v>
@@ -18724,7 +18825,9 @@
       <c r="I50" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J50" s="33"/>
+      <c r="J50" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K50" s="34" t="s">
         <v>569</v>
       </c>
@@ -18773,7 +18876,9 @@
       <c r="I51" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J51" s="33"/>
+      <c r="J51" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K51" s="34" t="s">
         <v>569</v>
       </c>
@@ -18822,7 +18927,9 @@
       <c r="I52" s="33" t="s">
         <v>937</v>
       </c>
-      <c r="J52" s="33"/>
+      <c r="J52" s="33" t="s">
+        <v>937</v>
+      </c>
       <c r="K52" s="34" t="s">
         <v>569</v>
       </c>
@@ -18871,7 +18978,9 @@
       <c r="I53" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J53" s="29"/>
+      <c r="J53" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K53" s="14"/>
       <c r="L53" s="14"/>
       <c r="M53" s="11" t="s">
@@ -18916,7 +19025,9 @@
       <c r="I54" s="29" t="s">
         <v>937</v>
       </c>
-      <c r="J54" s="29"/>
+      <c r="J54" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K54" s="14" t="s">
         <v>570</v>
       </c>
@@ -18961,7 +19072,9 @@
       <c r="I55" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J55" s="29"/>
+      <c r="J55" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K55" s="14" t="s">
         <v>570</v>
       </c>
@@ -19008,7 +19121,9 @@
       <c r="I56" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J56" s="29"/>
+      <c r="J56" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K56" s="14"/>
       <c r="L56" s="14"/>
       <c r="M56" s="11" t="s">
@@ -19053,7 +19168,9 @@
       <c r="I57" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J57" s="29"/>
+      <c r="J57" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
       <c r="M57" s="11" t="s">
@@ -19096,7 +19213,9 @@
       <c r="I58" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J58" s="29"/>
+      <c r="J58" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K58" s="14"/>
       <c r="L58" s="14"/>
       <c r="M58" s="11" t="s">
@@ -19141,7 +19260,9 @@
       <c r="I59" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J59" s="29"/>
+      <c r="J59" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K59" s="14"/>
       <c r="L59" s="14"/>
       <c r="M59" s="11" t="s">
@@ -19186,7 +19307,9 @@
       <c r="I60" s="29" t="s">
         <v>938</v>
       </c>
-      <c r="J60" s="29"/>
+      <c r="J60" s="29" t="s">
+        <v>938</v>
+      </c>
       <c r="K60" s="14"/>
       <c r="L60" s="14"/>
       <c r="M60" s="11" t="s">

</xml_diff>